<commit_message>
chore: remove temporary Excel files from data and exports directories
</commit_message>
<xml_diff>
--- a/data/Vaciado_ENAPROCE2026.xlsx
+++ b/data/Vaciado_ENAPROCE2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cristina.sanchez\Documents\VALIDADOR_VECTORES\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\martin.macias\Downloads\VALIDACION_VECTORES\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E688B70-A372-4608-9486-8425D53D1B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A40EAA8D-C8E0-4DA3-B042-D81F62080D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3394" uniqueCount="835">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3392" uniqueCount="835">
   <si>
     <t>ID_MUESTRA</t>
   </si>
@@ -2551,7 +2551,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -2562,6 +2562,14 @@
     <font>
       <sz val="11"/>
       <name val="Dialog"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2590,7 +2598,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -2603,6 +2611,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6911,8 +6920,8 @@
       <c r="U6" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="V6" s="5" t="s">
-        <v>601</v>
+      <c r="V6" s="7">
+        <v>1</v>
       </c>
       <c r="W6" s="5" t="s">
         <v>601</v>
@@ -6920,8 +6929,8 @@
       <c r="X6" s="5" t="s">
         <v>595</v>
       </c>
-      <c r="Y6" s="5" t="s">
-        <v>588</v>
+      <c r="Y6" s="7">
+        <v>1</v>
       </c>
       <c r="Z6" s="5" t="s">
         <v>590</v>
@@ -10131,6 +10140,7 @@
       <c r="T10" s="5" t="s">
         <v>595</v>
       </c>
+      <c r="U10" s="8"/>
       <c r="V10" s="5" t="s">
         <v>596</v>
       </c>

</xml_diff>